<commit_message>
Full first draft at pre-workflow QC.
</commit_message>
<xml_diff>
--- a/sewer/resources/watchdb.all_tables.xlsx
+++ b/sewer/resources/watchdb.all_tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11023"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/dev/watch-wv/sewer/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2757E5DE-3730-A64F-A24E-624780365826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E179A7D3-AC79-8940-9C41-AB0E48C466E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15180" yWindow="3720" windowWidth="30240" windowHeight="18980" activeTab="3" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
@@ -1947,12 +1947,6 @@
     <t>Influenza Virus B (NEP/NS1)</t>
   </si>
   <si>
-    <t>Human Norovirus GI (ORF1_2)</t>
-  </si>
-  <si>
-    <t>Human Norovirus GII (ORF1_2)</t>
-  </si>
-  <si>
     <t>SARS-CoV-2 (N2)</t>
   </si>
   <si>
@@ -2016,9 +2010,6 @@
     <t>Measles</t>
   </si>
   <si>
-    <t>Measles Virus, Wild Type (Unk)</t>
-  </si>
-  <si>
     <t>Measles Virus, Vaccine Strain (Unk)</t>
   </si>
   <si>
@@ -2035,6 +2026,15 @@
   </si>
   <si>
     <t>Bordetella pertussis</t>
+  </si>
+  <si>
+    <t>Norovirus GI, Human (ORF1_2)</t>
+  </si>
+  <si>
+    <t>Norovirus GII, Human (ORF1_2)</t>
+  </si>
+  <si>
+    <t>Measles Virus, Wild-Type (M)</t>
   </si>
 </sst>
 </file>
@@ -10645,16 +10645,16 @@
         <v>631</v>
       </c>
       <c r="D1" s="74" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="E1" s="74" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="F1" s="74" t="s">
         <v>375</v>
       </c>
       <c r="G1" s="74" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -10682,7 +10682,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="73" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B3" s="37" t="s">
         <v>561</v>
@@ -10705,7 +10705,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="73" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B4" s="37" t="s">
         <v>562</v>
@@ -10743,7 +10743,7 @@
         <v>377</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="G5" s="37" t="s">
         <v>376</v>
@@ -10766,7 +10766,7 @@
         <v>377</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="G6" s="37" t="s">
         <v>376</v>
@@ -10774,13 +10774,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="73" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B7" s="37" t="s">
         <v>382</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="D7" s="37" t="s">
         <v>392</v>
@@ -10797,13 +10797,13 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="73" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C8" s="73" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D8" s="37" t="s">
         <v>392</v>
@@ -10812,7 +10812,7 @@
         <v>377</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="G8" s="37" t="s">
         <v>376</v>
@@ -10820,13 +10820,13 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="37" t="s">
+        <v>657</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>658</v>
+      </c>
+      <c r="C9" s="37" t="s">
         <v>660</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>661</v>
-      </c>
-      <c r="C9" s="37" t="s">
-        <v>663</v>
       </c>
       <c r="D9" s="37" t="s">
         <v>393</v>
@@ -10835,7 +10835,7 @@
         <v>377</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="G9" s="37" t="s">
         <v>376</v>
@@ -10843,7 +10843,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="73" t="s">
-        <v>634</v>
+        <v>661</v>
       </c>
       <c r="B10" s="37" t="s">
         <v>571</v>
@@ -10866,7 +10866,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="73" t="s">
-        <v>635</v>
+        <v>662</v>
       </c>
       <c r="B11" s="37" t="s">
         <v>391</v>
@@ -10889,10 +10889,10 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="73" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="C12" s="73" t="s">
         <v>530</v>
@@ -10904,7 +10904,7 @@
         <v>377</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="G12" s="37" t="s">
         <v>381</v>
@@ -10912,7 +10912,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="73" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="B13" s="37" t="s">
         <v>385</v>
@@ -10935,7 +10935,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="73" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="B14" s="37" t="s">
         <v>388</v>
@@ -10958,13 +10958,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="73" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="B15" s="37" t="s">
         <v>389</v>
       </c>
       <c r="C15" s="73" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="D15" s="37" t="s">
         <v>392</v>
@@ -10976,21 +10976,21 @@
         <v>389</v>
       </c>
       <c r="G15" s="37" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="73" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="C16" s="73" t="s">
         <v>558</v>
       </c>
       <c r="D16" s="37" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E16" s="37" t="s">
         <v>315</v>
@@ -10999,18 +10999,18 @@
         <v>315</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="37" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="C17" s="37" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D17" s="37" t="s">
         <v>392</v>
@@ -11019,10 +11019,10 @@
         <v>377</v>
       </c>
       <c r="F17" s="37" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="G17" s="37" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
     </row>
   </sheetData>

</xml_diff>